<commit_message>
Add Rewards Hub winner selection
</commit_message>
<xml_diff>
--- a/uploads/1773465140866-Eltham Konnect Rate Sheet.xlsx
+++ b/uploads/1773465140866-Eltham Konnect Rate Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ea8ac7e28141b3d9/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramon\OneDrive\Desktop\ElthamKonnectSystem\backend\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25C72C46-6909-4DC6-B9AB-801634EEC4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A146E2F-1C0E-4686-8846-05B018E2A9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -413,7 +413,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>800</v>
+        <v>900</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -421,7 +421,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1100</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -429,7 +429,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1500</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -437,7 +437,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>1800</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -445,7 +445,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>2200</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -453,7 +453,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2600</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -461,7 +461,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>2900</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -469,7 +469,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>3300</v>
+        <v>3400</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -477,7 +477,7 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>3700</v>
+        <v>3800</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -485,7 +485,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>4200</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -493,7 +493,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>4500</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -501,7 +501,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>4800</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -509,7 +509,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>5100</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -517,7 +517,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>5400</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -525,7 +525,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>5700</v>
+        <v>5800</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -533,7 +533,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>6000</v>
+        <v>6100</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -541,7 +541,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>6300</v>
+        <v>6400</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -549,7 +549,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>6600</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -557,7 +557,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>6900</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -565,7 +565,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>7200</v>
+        <v>7300</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -573,7 +573,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>7350</v>
+        <v>7450</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +581,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>7450</v>
+        <v>7550</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -589,7 +589,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>7600</v>
+        <v>7700</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -597,7 +597,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>7750</v>
+        <v>7900</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -605,7 +605,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>7900</v>
+        <v>8100</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -613,7 +613,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>8150</v>
+        <v>8300</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -621,7 +621,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>8300</v>
+        <v>8500</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -629,7 +629,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>8450</v>
+        <v>8650</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -637,7 +637,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>8600</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -645,7 +645,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>8800</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -653,7 +653,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>11500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -661,7 +661,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>12000</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -669,7 +669,7 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>12500</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -677,7 +677,7 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>13000</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -685,7 +685,7 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>13500</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -693,7 +693,7 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>14000</v>
+        <v>14500</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -701,7 +701,7 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>14500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -709,7 +709,7 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>15000</v>
+        <v>15500</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -717,7 +717,7 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>15500</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -725,7 +725,7 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>16000</v>
+        <v>16500</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -733,7 +733,7 @@
         <v>41</v>
       </c>
       <c r="B42">
-        <v>16300</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -741,7 +741,7 @@
         <v>42</v>
       </c>
       <c r="B43">
-        <v>16500</v>
+        <v>17500</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -749,7 +749,7 @@
         <v>43</v>
       </c>
       <c r="B44">
-        <v>16800</v>
+        <v>18500</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -757,7 +757,7 @@
         <v>44</v>
       </c>
       <c r="B45">
-        <v>17200</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -765,7 +765,7 @@
         <v>45</v>
       </c>
       <c r="B46">
-        <v>17500</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -773,7 +773,7 @@
         <v>46</v>
       </c>
       <c r="B47">
-        <v>17800</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -781,7 +781,7 @@
         <v>47</v>
       </c>
       <c r="B48">
-        <v>18400</v>
+        <v>20400</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -789,7 +789,7 @@
         <v>48</v>
       </c>
       <c r="B49">
-        <v>18800</v>
+        <v>20700</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -797,7 +797,7 @@
         <v>49</v>
       </c>
       <c r="B50">
-        <v>19200</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -805,7 +805,7 @@
         <v>50</v>
       </c>
       <c r="B51">
-        <v>19600</v>
+        <v>21500</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -813,7 +813,7 @@
         <v>51</v>
       </c>
       <c r="B52">
-        <v>20000</v>
+        <v>21700</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -821,7 +821,7 @@
         <v>52</v>
       </c>
       <c r="B53">
-        <v>20400</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -829,7 +829,7 @@
         <v>53</v>
       </c>
       <c r="B54">
-        <v>20800</v>
+        <v>22300</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -837,7 +837,7 @@
         <v>54</v>
       </c>
       <c r="B55">
-        <v>21200</v>
+        <v>22600</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -845,7 +845,7 @@
         <v>55</v>
       </c>
       <c r="B56">
-        <v>21600</v>
+        <v>22900</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -853,7 +853,7 @@
         <v>56</v>
       </c>
       <c r="B57">
-        <v>22000</v>
+        <v>23300</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -861,7 +861,7 @@
         <v>57</v>
       </c>
       <c r="B58">
-        <v>22400</v>
+        <v>23700</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -869,7 +869,7 @@
         <v>58</v>
       </c>
       <c r="B59">
-        <v>22800</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -877,7 +877,7 @@
         <v>59</v>
       </c>
       <c r="B60">
-        <v>23200</v>
+        <v>24200</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -885,7 +885,7 @@
         <v>60</v>
       </c>
       <c r="B61">
-        <v>23600</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -893,7 +893,7 @@
         <v>61</v>
       </c>
       <c r="B62">
-        <v>23850</v>
+        <v>24900</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -901,7 +901,7 @@
         <v>62</v>
       </c>
       <c r="B63">
-        <v>24200</v>
+        <v>25300</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -909,7 +909,7 @@
         <v>63</v>
       </c>
       <c r="B64">
-        <v>24600</v>
+        <v>25700</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -917,7 +917,7 @@
         <v>64</v>
       </c>
       <c r="B65">
-        <v>24900</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -925,7 +925,7 @@
         <v>65</v>
       </c>
       <c r="B66">
-        <v>25300</v>
+        <v>26500</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -933,7 +933,7 @@
         <v>66</v>
       </c>
       <c r="B67">
-        <v>25600</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -941,7 +941,7 @@
         <v>67</v>
       </c>
       <c r="B68">
-        <v>25900</v>
+        <v>27300</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -949,7 +949,7 @@
         <v>68</v>
       </c>
       <c r="B69">
-        <v>26300</v>
+        <v>27700</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -957,7 +957,7 @@
         <v>69</v>
       </c>
       <c r="B70">
-        <v>26700</v>
+        <v>28100</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -965,7 +965,7 @@
         <v>70</v>
       </c>
       <c r="B71">
-        <v>27200</v>
+        <v>28600</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -973,7 +973,7 @@
         <v>71</v>
       </c>
       <c r="B72">
-        <v>27600</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -981,7 +981,7 @@
         <v>72</v>
       </c>
       <c r="B73">
-        <v>27900</v>
+        <v>29500</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -989,7 +989,7 @@
         <v>73</v>
       </c>
       <c r="B74">
-        <v>28400</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -997,7 +997,7 @@
         <v>74</v>
       </c>
       <c r="B75">
-        <v>28800</v>
+        <v>30300</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -1005,7 +1005,7 @@
         <v>75</v>
       </c>
       <c r="B76">
-        <v>29200</v>
+        <v>30700</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -1013,7 +1013,7 @@
         <v>76</v>
       </c>
       <c r="B77">
-        <v>29600</v>
+        <v>31100</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -1021,7 +1021,7 @@
         <v>77</v>
       </c>
       <c r="B78">
-        <v>29900</v>
+        <v>31350</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -1029,7 +1029,7 @@
         <v>78</v>
       </c>
       <c r="B79">
-        <v>30200</v>
+        <v>31700</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -1037,7 +1037,7 @@
         <v>79</v>
       </c>
       <c r="B80">
-        <v>30600</v>
+        <v>31950</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -1045,7 +1045,7 @@
         <v>80</v>
       </c>
       <c r="B81">
-        <v>30900</v>
+        <v>33350</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -1053,7 +1053,7 @@
         <v>81</v>
       </c>
       <c r="B82">
-        <v>31300</v>
+        <v>33700</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -1061,7 +1061,7 @@
         <v>82</v>
       </c>
       <c r="B83">
-        <v>31600</v>
+        <v>33900</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -1069,7 +1069,7 @@
         <v>83</v>
       </c>
       <c r="B84">
-        <v>32000</v>
+        <v>34200</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -1077,7 +1077,7 @@
         <v>84</v>
       </c>
       <c r="B85">
-        <v>32600</v>
+        <v>34400</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -1085,7 +1085,7 @@
         <v>85</v>
       </c>
       <c r="B86">
-        <v>33000</v>
+        <v>34600</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -1093,7 +1093,7 @@
         <v>86</v>
       </c>
       <c r="B87">
-        <v>33400</v>
+        <v>34800</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -1101,7 +1101,7 @@
         <v>87</v>
       </c>
       <c r="B88">
-        <v>33800</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -1109,7 +1109,7 @@
         <v>88</v>
       </c>
       <c r="B89">
-        <v>34200</v>
+        <v>35200</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -1117,7 +1117,7 @@
         <v>89</v>
       </c>
       <c r="B90">
-        <v>34600</v>
+        <v>35400</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -1125,7 +1125,7 @@
         <v>90</v>
       </c>
       <c r="B91">
-        <v>35000</v>
+        <v>35600</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -1133,7 +1133,7 @@
         <v>91</v>
       </c>
       <c r="B92">
-        <v>35300</v>
+        <v>35800</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -1141,7 +1141,7 @@
         <v>92</v>
       </c>
       <c r="B93">
-        <v>35700</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -1149,7 +1149,7 @@
         <v>93</v>
       </c>
       <c r="B94">
-        <v>36000</v>
+        <v>36200</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix updated rates calculator syntax
</commit_message>
<xml_diff>
--- a/uploads/1773465140866-Eltham Konnect Rate Sheet.xlsx
+++ b/uploads/1773465140866-Eltham Konnect Rate Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramon\OneDrive\Desktop\ElthamKonnectSystem\backend\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A146E2F-1C0E-4686-8846-05B018E2A9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CC40AE-AE08-4753-880A-53972A23AE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -493,7 +493,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>4600</v>
+        <v>4700</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -501,7 +501,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>4900</v>
+        <v>5100</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -509,7 +509,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>5200</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -517,7 +517,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>5500</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -525,7 +525,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>5800</v>
+        <v>6300</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -533,7 +533,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>6100</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -541,7 +541,7 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>6400</v>
+        <v>7100</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -549,7 +549,7 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>6700</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -557,7 +557,7 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>7000</v>
+        <v>7900</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -565,7 +565,7 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>7300</v>
+        <v>8300</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -573,7 +573,7 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>7450</v>
+        <v>8550</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +581,7 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>7550</v>
+        <v>8900</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -589,7 +589,7 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>7700</v>
+        <v>9400</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -597,7 +597,7 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>7900</v>
+        <v>9900</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -605,7 +605,7 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>8100</v>
+        <v>10200</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -613,7 +613,7 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>8300</v>
+        <v>10600</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -621,7 +621,7 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>8500</v>
+        <v>10900</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -629,7 +629,7 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>8650</v>
+        <v>11300</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -637,7 +637,7 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>8800</v>
+        <v>11600</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -645,7 +645,7 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>9200</v>
+        <v>11900</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -653,7 +653,7 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>12000</v>
+        <v>12400</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -661,7 +661,7 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>12500</v>
+        <v>12800</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>